<commit_message>
fix(onboarding): rebuild instruction register workbook
</commit_message>
<xml_diff>
--- a/templates/registers/instruction_register_template.xlsx
+++ b/templates/registers/instruction_register_template.xlsx
@@ -13,7 +13,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="role_matrix" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="examples" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'instruction_log'!$A$1:$P$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'instruction_catalog'!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'role_matrix'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'examples'!$A$1:$F$5</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -31,9 +37,10 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -42,11 +49,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -54,16 +66,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7B7B7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -140,6 +169,86 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_README" displayName="tbl_README" ref="A1:B6" headerRowCount="1">
+  <autoFilter ref="A1:B6"/>
+  <tableColumns count="2">
+    <tableColumn id="1" name="Раздел"/>
+    <tableColumn id="2" name="Описание"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_instruction_log" displayName="tbl_instruction_log" ref="A1:P5" headerRowCount="1">
+  <autoFilter ref="A1:P5"/>
+  <tableColumns count="16">
+    <tableColumn id="1" name="N"/>
+    <tableColumn id="2" name="Дата инструктажа"/>
+    <tableColumn id="3" name="ФИО сотрудника"/>
+    <tableColumn id="4" name="Табельный номер"/>
+    <tableColumn id="5" name="Подразделение"/>
+    <tableColumn id="6" name="Должность"/>
+    <tableColumn id="7" name="Вид инструктажа"/>
+    <tableColumn id="8" name="Название/код инструкции"/>
+    <tableColumn id="9" name="Основание/программа"/>
+    <tableColumn id="10" name="Инструктирующий"/>
+    <tableColumn id="11" name="Должность инструктирующего"/>
+    <tableColumn id="12" name="Результат проверки знаний"/>
+    <tableColumn id="13" name="Подпись инструктируемого"/>
+    <tableColumn id="14" name="Подпись инструктирующего"/>
+    <tableColumn id="15" name="Следующий инструктаж"/>
+    <tableColumn id="16" name="Примечание"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tbl_instruction_catalog" displayName="tbl_instruction_catalog" ref="A1:F8" headerRowCount="1">
+  <autoFilter ref="A1:F8"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="Код инструкции"/>
+    <tableColumn id="2" name="Название"/>
+    <tableColumn id="3" name="Категория"/>
+    <tableColumn id="4" name="Для каких ролей"/>
+    <tableColumn id="5" name="Периодичность/триггер"/>
+    <tableColumn id="6" name="Ответственный"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbl_role_matrix" displayName="tbl_role_matrix" ref="A1:E6" headerRowCount="1">
+  <autoFilter ref="A1:E6"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Роль"/>
+    <tableColumn id="2" name="Формат/объект"/>
+    <tableColumn id="3" name="Обязательные инструктажи"/>
+    <tableColumn id="4" name="Дополнительные проверки"/>
+    <tableColumn id="5" name="Комментарий"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tbl_examples" displayName="tbl_examples" ref="A1:F5" headerRowCount="1">
+  <autoFilter ref="A1:F5"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="Сценарий"/>
+    <tableColumn id="2" name="Сотрудник"/>
+    <tableColumn id="3" name="Роль"/>
+    <tableColumn id="4" name="Инструктажи"/>
+    <tableColumn id="5" name="Статус"/>
+    <tableColumn id="6" name="Комментарий"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -431,63 +540,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>??????????</t>
+          <t>Раздел</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Public-safe ?????? ????? ???????????? ??? onboarding-??????.</t>
+          <t>Описание</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>??????????????</t>
+          <t>Назначение</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>??? ?????? ????????; ?? ??????????? ???????? ???, ???????, ????????, ????????, ???????? ? ?????? ????.</t>
+          <t>Public-safe шаблон книги учета инструктажей для onboarding-агента.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>????????</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>???? ?????? ??????, ?? ???????? ?????? ????????? ?????.</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Предупреждение</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Все данные синтетические. Не вставлять реальные ФИО, табельные номера, подписи, кабинеты, пропуска, телефоны, email, IP и маршруты доступа.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>????????</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>????? ??????????? ??????????? ????? ? HR, ??, ?? ? ?????????????? ?? ??????.</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Правила</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Книгу можно использовать как структуру журнала, но реальные журналы и формулировки должны быть проверены HR, ОТ, ИБ и ответственными за процесс.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Листы</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>instruction_log — журнал; instruction_catalog — каталог инструкций; role_matrix — связь ролей с инструктажами; examples — короткие synthetic сценарии.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Файл не подтверждает обучение, не выдает допуски и не заменяет официальные журналы инструктажей.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -497,25 +634,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="27" customWidth="1" min="12" max="12"/>
+    <col width="29" customWidth="1" min="12" max="12"/>
     <col width="26" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="37" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -526,242 +663,406 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>???? ???????????</t>
+          <t>Дата инструктажа</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>??? ??????????</t>
+          <t>ФИО сотрудника</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>????????? ?????</t>
+          <t>Табельный номер</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>?????????????</t>
+          <t>Подразделение</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>?????????</t>
+          <t>Должность</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>??? ???????????</t>
+          <t>Вид инструктажа</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>????????/??? ??????????</t>
+          <t>Название/код инструкции</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>?????????/?????????</t>
+          <t>Основание/программа</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>???????????????</t>
+          <t>Инструктирующий</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>????????? ????????????????</t>
+          <t>Должность инструктирующего</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>????????? ???????? ??????</t>
+          <t>Результат проверки знаний</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>??????? ????????????????</t>
+          <t>Подпись инструктируемого</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>??????? ????????????????</t>
+          <t>Подпись инструктирующего</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>????????? ??????????</t>
+          <t>Следующий инструктаж</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>??????????</t>
+          <t>Примечание</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>???????? ???? ????????</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Примеров Петр Петрович</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>TEST-0001</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>TEST-DEPARTMENT</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>??????? TEST-APP</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>???????</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>инженер тестовой команды</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>вводный</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>OT-INTRO-TEST</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>TEST-PROGRAM</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>?????????? ????????</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>?????????? ??</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>????????</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Инструктор Тестовый</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>специалист ОТ</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>пройдено</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>synthetic-signature</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>synthetic-signature</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>??????</t>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>пример</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>??????? ???? ?????????</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Тестова Анна Сергеевна</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>TEST-0002</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>TEST-DEPARTMENT</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>???????? TEST-BI</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>FIRE-TEST</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>TEST-FIRE-PROGRAM</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>?????????? ????????</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>????????????? ?? ??</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>????????</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>аналитик TEST-BI</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>ПВТР</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>PVTR-TEST</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>TEST-PVTR-PROGRAM</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>HR Тестовый</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>HR business partner</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>пройдено</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>synthetic-signature</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>synthetic-signature</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>??????</t>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>пример</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Образцов Илья Романович</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>TEST-0003</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>TEST-FIELD</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>инженер выездной группы</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>первичный</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>FIELD-ELECTRIC-TEST</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>TEST-FIELD-PROGRAM</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Инструктор Полевой</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>ответственный за работы</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>требует профильной проверки</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>synthetic-signature</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>synthetic-signature</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>пример для роли с повышенным риском</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Макетова Мария Олеговна</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>TEST-0004</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>TEST-IT</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>администратор тестовой среды</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>ИБ/ЛВС</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>IB-LAN-TEST</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>TEST-IB-PROGRAM</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Инструктор ИБ</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>специалист ИБ</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>пройдено</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>synthetic-signature</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>synthetic-signature</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>пример без реальных доступов</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:P5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -771,211 +1072,279 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>??? ??????????</t>
+          <t>Код инструкции</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>????????</t>
+          <t>Название</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>?????????</t>
+          <t>Категория</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>??? ????? ?????</t>
+          <t>Для каких ролей</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>?????????????/???????</t>
+          <t>Периодичность/триггер</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>?????????????</t>
+          <t>Ответственный</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>PVTR-TEST</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>???????????? ? ????</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>????</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>??? ??????????</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>??? ?????? ? ??????????</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Правила внутреннего трудового распорядка</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>ПВТР</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>все сотрудники</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>при приеме и изменениях</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>OT-INTRO-TEST</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>??????? ?????????? ?? ??</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>?????? ?????</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>??? ??????????</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>??? ??????</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>?????????? ??</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Вводный инструктаж по охране труда</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>охрана труда</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>все сотрудники</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>при приеме</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>специалист ОТ</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>FIRE-TEST</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>??????????????? ??????????</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>???????? ????????????</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>??? ??????????</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>?? ????????? ????????</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>????????????? ?? ??</t>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Инструктаж по пожарной безопасности</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>пожарная безопасность</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>все сотрудники</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>по локальному графику</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>ответственный за ПБ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>FIRST-AID-TEST</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Первая помощь: базовые действия</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>первая помощь</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>офисные и выездные сотрудники</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>при приеме и по графику</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>специалист ОТ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>IB-LAN-TEST</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>??????? ??? ? ??</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>?????????? ? ??-????????</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>??? ?????? ???????</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>?? / IT</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Правила ЛВС и информационной безопасности</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>ИБ</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>офисные и IT-сотрудники</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>при выдаче доступа</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>ИБ / IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>FIELD-ELECTRIC-TEST</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>?????? ? ?????????????????</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>?????????? ??????</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>???????? ????</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>??????? ?????????? ????????</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>?????????? ????????????</t>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Работы в электроустановках</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>повышенный риск</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>выездные роли</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>требует профильной проверки</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>ответственный руководитель</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>HEIGHT-WORK-TEST</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Работы на высоте</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>повышенный риск</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>выездные роли</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>требует профильной проверки</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>ответственный руководитель</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -985,153 +1354,184 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>????</t>
+          <t>Роль</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>????/????????/?????</t>
+          <t>Формат/объект</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>???????????? ???????????</t>
+          <t>Обязательные инструктажи</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>?????????????? ???????</t>
+          <t>Дополнительные проверки</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>???????????</t>
+          <t>Комментарий</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>??????? ??-?????????</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>????</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>????; ??; ??; ???/??; ????????????; ???????</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>??? ?? ?????????</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>???????? ? ????? ?? ??????</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>офисный сотрудник</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>офис</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>ПВТР; ОТ; ПБ; первая помощь; ЛВС/ИБ</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>пропуск; кабинет/ключи; имущество</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>использовать только TEST-данные</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>????????? ??-?????????</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>????????</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>????; ??; ??; ???/??; ????????????</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>??? ?? ?????????</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>?????????? ?????? ?? ???????</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>удаленный сотрудник</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>удаленно</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>ПВТР; ОТ; ПБ; ЛВС/ИБ</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>оборудование; удаленный доступ</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>без кабинетов и пропусков</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>???????? ?????????????? ?????????</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>?????</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>????; ??; ??; ?????? ??????; ???/??; ????????????</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>????????????????; ??????</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>??????? ?????????? ????????</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>IT-инженер</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>офис/удаленно</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ПВТР; ОТ; ПБ; первая помощь; ЛВС/ИБ</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>доступы к тестовым системам</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>не указывать секреты и токены</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>?????????</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>??????/????</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>????; ??; ???/??; ???????</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>?? ???????? ? ???????</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>???? ??????? ?????????</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>инженер выездной группы</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>выезд</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>ПВТР; ОТ; ПБ; первая помощь; полевой инструктаж</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>электроустановки; высота</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>требует профильной проверки</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>подрядчик</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>офис/выезд</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>ПВТР; ПБ; ЛВС/ИБ; локальные правила объекта</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>срок доступа; сопровождающий</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>доступ только по согласованию</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1141,146 +1541,182 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>????????</t>
+          <t>Сценарий</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>?????????</t>
+          <t>Сотрудник</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>????</t>
+          <t>Роль</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>?????????</t>
+          <t>Инструктажи</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>??????</t>
+          <t>Статус</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>???????????</t>
+          <t>Комментарий</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>office</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>???????? ???? ????????</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>??????? TEST-APP</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>????; ??; ??; ???/??</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>????? ???????</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>??? ???????? ??????</t>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Примеров Петр Петрович</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>инженер TEST-APP</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>ПВТР; ОТ; ПБ; ЛВС/ИБ</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>можно готовить пакет</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>без реальных кабинетов</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>remote</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>??????? ???? ?????????</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>???????? TEST-BI</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>????; ??; ??; ???/??</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>????? ???????</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>??? ??????????? ???????</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Тестова Анна Сергеевна</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>аналитик TEST-BI</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ПВТР; ОТ; ПБ; ЛВС/ИБ</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>можно готовить пакет</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>без физического доступа</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>field</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>???????? ???? ?????????</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>???????? ??????? TEST-GRID</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>????; ??; ??; ????????????????; ??????</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>??????? ?????????? ????????</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>?????? ?? ????? ???????</t>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Образцов Илья Романович</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>инженер выездной группы</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>ПВТР; ОТ; ПБ; полевой; электроустановки</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>требует профильной проверки</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>не выдавать допуск автоматически</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>contractor</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Макетова Мария Олеговна</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>подрядчик TEST-VENDOR</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>ПВТР; ПБ; ЛВС/ИБ; локальные правила объекта</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>требует согласования</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>срок доступа ограничен</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(onboarding): clean public onboarding kit
- Rewrite README and PLAN as user-facing instructions
- Remove publication and synthetic wording from prompts, templates, examples, and employee packages
- Update instruction register workbook text and user-facing launch guidance

Co-Authored-By: AI Agent <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/templates/registers/instruction_register_template.xlsx
+++ b/templates/registers/instruction_register_template.xlsx
@@ -567,7 +567,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Синтетический шаблон книги учета инструктажей для onboarding-агента.</t>
+          <t>Шаблон книги учета инструктажей для onboarding-агента.</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Все данные синтетические. Не вставлять реальные ФИО, табельные номера, подписи, кабинеты, пропуска, телефоны, email, IP и маршруты доступа.</t>
+          <t>Перед применением согласуйте состав листов, программы инструктажей и форму подписи с HR, ОТ, ИБ и ответственными за процесс.</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>instruction_log — журнал; instruction_catalog — каталог инструкций; role_matrix — связь ролей с инструктажами; examples — короткие synthetic сценарии.</t>
+          <t>instruction_log — журнал; instruction_catalog — каталог инструкций; role_matrix — связь ролей с инструктажами; examples — короткие рабочие сценарии.</t>
         </is>
       </c>
     </row>
@@ -798,12 +798,12 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>synthetic-signature</t>
+          <t>[подпись]</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>synthetic-signature</t>
+          <t>[подпись]</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -878,12 +878,12 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>synthetic-signature</t>
+          <t>[подпись]</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>synthetic-signature</t>
+          <t>[подпись]</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
@@ -958,12 +958,12 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>synthetic-signature</t>
+          <t>[подпись]</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>synthetic-signature</t>
+          <t>[подпись]</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
@@ -1038,12 +1038,12 @@
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>synthetic-signature</t>
+          <t>[подпись]</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>synthetic-signature</t>
+          <t>[подпись]</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">

</xml_diff>